<commit_message>
ajustado erro na coluna da acuracia
</commit_message>
<xml_diff>
--- a/datasets/metricas.xlsx
+++ b/datasets/metricas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,7 +434,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Acuracia</t>
+          <t>Acurácia</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -450,11 +450,6 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>Precisao</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Acurácia</t>
         </is>
       </c>
     </row>
@@ -469,7 +464,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -478,9 +473,6 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -495,7 +487,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -504,9 +496,6 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -521,7 +510,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -530,9 +519,6 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -547,7 +533,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -556,9 +542,6 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -573,7 +556,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -582,9 +565,6 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>